<commit_message>
Implement strict NIP-based Dosen PA system - Store dosen username/NIP instead of name in nama_dosen_pa and dosen_pa columns - Add model relations and display helpers - Update all queries to use NIP - Add backfill command and regression tests - All 103 tests passing
</commit_message>
<xml_diff>
--- a/public/templates/Format_Import_Akun.xlsx
+++ b/public/templates/Format_Import_Akun.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="12">
   <si>
     <t>Nama Lengkap</t>
   </si>
@@ -29,7 +29,7 @@
     <t>Role</t>
   </si>
   <si>
-    <t>Nama Dosen PA</t>
+    <t>NIP Dosen PA</t>
   </si>
   <si>
     <t>Jenis Magang</t>
@@ -45,9 +45,6 @@
   </si>
   <si>
     <t>mahasiswa</t>
-  </si>
-  <si>
-    <t>Pak Dosen</t>
   </si>
   <si>
     <t>Magang</t>
@@ -412,13 +409,13 @@
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="21.138" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="13.997" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="11.711" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="16.425" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="10.569" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="15.282" customWidth="true" style="0"/>
+    <col min="2" max="2" width="21.138" customWidth="true" style="0"/>
+    <col min="3" max="3" width="13.997" customWidth="true" style="0"/>
+    <col min="4" max="4" width="11.711" customWidth="true" style="0"/>
+    <col min="5" max="5" width="16.425" customWidth="true" style="0"/>
+    <col min="6" max="6" width="15.282" customWidth="true" style="0"/>
+    <col min="7" max="7" width="10.569" customWidth="true" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -457,14 +454,14 @@
       <c r="D2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2">
+        <v>1234567890</v>
+      </c>
+      <c r="F2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>11</v>
-      </c>
-      <c r="G2" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>